<commit_message>
final simulations for arxiv
</commit_message>
<xml_diff>
--- a/experiments/batch_results_tomato2/results_summary.xlsx
+++ b/experiments/batch_results_tomato2/results_summary.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,119 +436,39 @@
         </is>
       </c>
       <c r="B1" s="1" t="n">
-        <v>0.004</v>
+        <v>0.002032</v>
       </c>
       <c r="C1" s="1" t="n">
-        <v>0.006</v>
+        <v>0.002794</v>
       </c>
       <c r="D1" s="1" t="n">
-        <v>0.008</v>
+        <v>0.003683</v>
       </c>
       <c r="E1" s="1" t="n">
-        <v>0.01</v>
+        <v>0.004572</v>
       </c>
       <c r="F1" s="1" t="n">
-        <v>0.012</v>
+        <v>0.005715</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="B2" t="n">
-        <v>0.004947626457087561</v>
+        <v>0.002509328578874172</v>
       </c>
       <c r="C2" t="n">
-        <v>0.007421232715282329</v>
+        <v>0.003450971480670393</v>
       </c>
       <c r="D2" t="n">
-        <v>0.009894765042940913</v>
+        <v>0.004549313089409017</v>
       </c>
       <c r="E2" t="n">
-        <v>0.01236826928272441</v>
+        <v>0.005647945579020548</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01484174397828714</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="n">
-        <v>0.004896470007774207</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.00734475105746963</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.009793351182586551</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.01224294055870168</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.01469104865116884</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.004936296293132103</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.007404373652032175</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.009872992079986827</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.01234128741778345</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.01480973683173561</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="B5" t="n">
-        <v>0.004922238865355949</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.007383936432169762</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.009846273899308646</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.01231015549390997</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.01478068383776372</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="B6" t="n">
-        <v>0.004946788948262479</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.007419426590994357</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.009892976121244845</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.01236955369971967</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.01484504890308261</v>
+        <v>0.007059915563942015</v>
       </c>
     </row>
   </sheetData>
@@ -562,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -572,119 +492,39 @@
         </is>
       </c>
       <c r="B1" s="1" t="n">
-        <v>0.004</v>
+        <v>0.002032</v>
       </c>
       <c r="C1" s="1" t="n">
-        <v>0.006</v>
+        <v>0.002794</v>
       </c>
       <c r="D1" s="1" t="n">
-        <v>0.008</v>
+        <v>0.003683</v>
       </c>
       <c r="E1" s="1" t="n">
-        <v>0.01</v>
+        <v>0.004572</v>
       </c>
       <c r="F1" s="1" t="n">
-        <v>0.012</v>
+        <v>0.005715</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7002707647583343</v>
+        <v>1.300069640420586</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7002708232811274</v>
+        <v>1.30006922682102</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7002709324541296</v>
+        <v>1.300069477492316</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7002711045530072</v>
+        <v>1.300069247991325</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7002712371304106</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="n">
-        <v>1.000154847805969</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1.000154838940415</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1.000154828413736</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1.000154827245867</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1.000154815403257</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>1.3000688883507</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1.300068958116634</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1.3000694384251</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1.300068907226196</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1.30006889603542</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="B5" t="n">
-        <v>1.600036371506295</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1.600036350550061</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1.60003636905414</v>
-      </c>
-      <c r="E5" t="n">
-        <v>1.600036362311439</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1.600037077032805</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="B6" t="n">
-        <v>1.900018294952052</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1.900018095222261</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1.900018423446048</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1.900021284664228</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1.900021287224129</v>
+        <v>1.300069212893259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>